<commit_message>
Compare Number and Percent values individually against the site, not summed totals
Rewrites the site trend check to match each row's exact location +
category + data format against that same series on the site, instead
of summing 'Number' values across breakdown categories into one
combined total. This lets 'Percent' values be checked too (previously
skipped entirely, since percentages aren't additive across
categories) - so a percent that's wrong because of a bad denominator
now gets flagged even when the number next to it is correct.
</commit_message>
<xml_diff>
--- a/data/CLEANED_3.6_PretermBirths_2023.xlsx
+++ b/data/CLEANED_3.6_PretermBirths_2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29711"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaitl\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a049744a5ceb6a/Documents/Every Texan/R/Kids Count Data Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAB30BCB-5F2E-4085-B77E-55A61A3D175C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{BAB30BCB-5F2E-4085-B77E-55A61A3D175C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E933DFA-7D34-4125-AF56-EF2F0ADDC4D3}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{78DDF658-3C05-42B1-92AA-6902B78F2627}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{78DDF658-3C05-42B1-92AA-6902B78F2627}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="8" r:id="rId1"/>
@@ -843,7 +843,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -898,6 +898,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1218,9 +1222,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CFF0B5D-6958-45BE-A874-CCEBECBB9950}">
   <dimension ref="A1:F511"/>
-  <sheetFormatPr defaultColWidth="17.28515625" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="17.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1240,7 +1244,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1260,7 +1264,7 @@
         <v>6515</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1280,7 +1284,7 @@
         <v>6515</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1300,7 +1304,7 @@
         <v>6516</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -1320,7 +1324,7 @@
         <v>6516</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1340,7 +1344,7 @@
         <v>6517</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1360,7 +1364,7 @@
         <v>6517</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1380,7 +1384,7 @@
         <v>6518</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -1400,7 +1404,7 @@
         <v>6518</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -1420,7 +1424,7 @@
         <v>6519</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1440,7 +1444,7 @@
         <v>6519</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -1460,7 +1464,7 @@
         <v>6520</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -1480,7 +1484,7 @@
         <v>6520</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -1500,7 +1504,7 @@
         <v>6521</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -1520,7 +1524,7 @@
         <v>6521</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -1540,7 +1544,7 @@
         <v>6522</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -1560,7 +1564,7 @@
         <v>6522</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -1580,7 +1584,7 @@
         <v>6523</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -1600,7 +1604,7 @@
         <v>6523</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -1620,7 +1624,7 @@
         <v>6524</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -1640,7 +1644,7 @@
         <v>6524</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>6</v>
       </c>
@@ -1660,7 +1664,7 @@
         <v>6525</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>6</v>
       </c>
@@ -1680,7 +1684,7 @@
         <v>6525</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>6</v>
       </c>
@@ -1700,7 +1704,7 @@
         <v>6526</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>6</v>
       </c>
@@ -1720,7 +1724,7 @@
         <v>6526</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>6</v>
       </c>
@@ -1740,7 +1744,7 @@
         <v>6527</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>6</v>
       </c>
@@ -1760,7 +1764,7 @@
         <v>6527</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>6</v>
       </c>
@@ -1780,7 +1784,7 @@
         <v>6528</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>6</v>
       </c>
@@ -1800,7 +1804,7 @@
         <v>6528</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>6</v>
       </c>
@@ -1820,7 +1824,7 @@
         <v>6529</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>6</v>
       </c>
@@ -1840,7 +1844,7 @@
         <v>6529</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>6</v>
       </c>
@@ -1860,7 +1864,7 @@
         <v>6530</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>6</v>
       </c>
@@ -1880,7 +1884,7 @@
         <v>6530</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>6</v>
       </c>
@@ -1900,7 +1904,7 @@
         <v>6531</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>6</v>
       </c>
@@ -1920,7 +1924,7 @@
         <v>6531</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>6</v>
       </c>
@@ -1940,7 +1944,7 @@
         <v>6532</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>6</v>
       </c>
@@ -1960,7 +1964,7 @@
         <v>6532</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>6</v>
       </c>
@@ -1980,7 +1984,7 @@
         <v>6533</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>6</v>
       </c>
@@ -2000,7 +2004,7 @@
         <v>6533</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>6</v>
       </c>
@@ -2020,7 +2024,7 @@
         <v>6534</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>6</v>
       </c>
@@ -2040,7 +2044,7 @@
         <v>6534</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>6</v>
       </c>
@@ -2060,7 +2064,7 @@
         <v>6535</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>6</v>
       </c>
@@ -2080,7 +2084,7 @@
         <v>6535</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>6</v>
       </c>
@@ -2100,7 +2104,7 @@
         <v>6536</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>6</v>
       </c>
@@ -2120,7 +2124,7 @@
         <v>6536</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>6</v>
       </c>
@@ -2140,7 +2144,7 @@
         <v>6537</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>6</v>
       </c>
@@ -2160,7 +2164,7 @@
         <v>6537</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>6</v>
       </c>
@@ -2180,7 +2184,7 @@
         <v>6538</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>6</v>
       </c>
@@ -2200,7 +2204,7 @@
         <v>6538</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>6</v>
       </c>
@@ -2220,7 +2224,7 @@
         <v>6539</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>6</v>
       </c>
@@ -2240,7 +2244,7 @@
         <v>6539</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>6</v>
       </c>
@@ -2260,7 +2264,7 @@
         <v>6540</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>6</v>
       </c>
@@ -2280,7 +2284,7 @@
         <v>6540</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>6</v>
       </c>
@@ -2300,7 +2304,7 @@
         <v>6541</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>6</v>
       </c>
@@ -2320,7 +2324,7 @@
         <v>6541</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>6</v>
       </c>
@@ -2340,7 +2344,7 @@
         <v>6542</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>6</v>
       </c>
@@ -2360,7 +2364,7 @@
         <v>6542</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>6</v>
       </c>
@@ -2380,7 +2384,7 @@
         <v>6543</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>6</v>
       </c>
@@ -2400,7 +2404,7 @@
         <v>6543</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>6</v>
       </c>
@@ -2420,7 +2424,7 @@
         <v>6544</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>6</v>
       </c>
@@ -2440,7 +2444,7 @@
         <v>6544</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>6</v>
       </c>
@@ -2460,7 +2464,7 @@
         <v>6545</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>6</v>
       </c>
@@ -2480,7 +2484,7 @@
         <v>6545</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>6</v>
       </c>
@@ -2500,7 +2504,7 @@
         <v>6546</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>6</v>
       </c>
@@ -2520,7 +2524,7 @@
         <v>6546</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>6</v>
       </c>
@@ -2540,7 +2544,7 @@
         <v>6547</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>6</v>
       </c>
@@ -2560,7 +2564,7 @@
         <v>6547</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>6</v>
       </c>
@@ -2580,7 +2584,7 @@
         <v>6548</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>6</v>
       </c>
@@ -2600,7 +2604,7 @@
         <v>6548</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>6</v>
       </c>
@@ -2620,7 +2624,7 @@
         <v>6549</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>6</v>
       </c>
@@ -2640,7 +2644,7 @@
         <v>6549</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>6</v>
       </c>
@@ -2660,7 +2664,7 @@
         <v>6550</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>6</v>
       </c>
@@ -2680,7 +2684,7 @@
         <v>6550</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>6</v>
       </c>
@@ -2700,7 +2704,7 @@
         <v>6551</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>6</v>
       </c>
@@ -2720,7 +2724,7 @@
         <v>6551</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>6</v>
       </c>
@@ -2740,7 +2744,7 @@
         <v>6552</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>6</v>
       </c>
@@ -2760,7 +2764,7 @@
         <v>6552</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>6</v>
       </c>
@@ -2780,7 +2784,7 @@
         <v>6553</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>6</v>
       </c>
@@ -2800,7 +2804,7 @@
         <v>6553</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>6</v>
       </c>
@@ -2820,7 +2824,7 @@
         <v>6554</v>
       </c>
     </row>
-    <row r="81" spans="1:6">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>6</v>
       </c>
@@ -2840,7 +2844,7 @@
         <v>6554</v>
       </c>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>6</v>
       </c>
@@ -2860,7 +2864,7 @@
         <v>6555</v>
       </c>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>6</v>
       </c>
@@ -2880,7 +2884,7 @@
         <v>6555</v>
       </c>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>6</v>
       </c>
@@ -2900,7 +2904,7 @@
         <v>6556</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>6</v>
       </c>
@@ -2920,7 +2924,7 @@
         <v>6556</v>
       </c>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>6</v>
       </c>
@@ -2940,7 +2944,7 @@
         <v>6557</v>
       </c>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>6</v>
       </c>
@@ -2960,7 +2964,7 @@
         <v>6557</v>
       </c>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>6</v>
       </c>
@@ -2980,7 +2984,7 @@
         <v>6558</v>
       </c>
     </row>
-    <row r="89" spans="1:6">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>6</v>
       </c>
@@ -3000,7 +3004,7 @@
         <v>6558</v>
       </c>
     </row>
-    <row r="90" spans="1:6">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>6</v>
       </c>
@@ -3020,7 +3024,7 @@
         <v>6559</v>
       </c>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>6</v>
       </c>
@@ -3040,7 +3044,7 @@
         <v>6559</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>6</v>
       </c>
@@ -3060,7 +3064,7 @@
         <v>6560</v>
       </c>
     </row>
-    <row r="93" spans="1:6">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>6</v>
       </c>
@@ -3080,7 +3084,7 @@
         <v>6560</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>6</v>
       </c>
@@ -3100,7 +3104,7 @@
         <v>6561</v>
       </c>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>6</v>
       </c>
@@ -3120,7 +3124,7 @@
         <v>6561</v>
       </c>
     </row>
-    <row r="96" spans="1:6">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>6</v>
       </c>
@@ -3140,7 +3144,7 @@
         <v>6562</v>
       </c>
     </row>
-    <row r="97" spans="1:6">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>6</v>
       </c>
@@ -3160,7 +3164,7 @@
         <v>6562</v>
       </c>
     </row>
-    <row r="98" spans="1:6">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>6</v>
       </c>
@@ -3180,7 +3184,7 @@
         <v>6563</v>
       </c>
     </row>
-    <row r="99" spans="1:6">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>6</v>
       </c>
@@ -3200,7 +3204,7 @@
         <v>6563</v>
       </c>
     </row>
-    <row r="100" spans="1:6">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>6</v>
       </c>
@@ -3220,7 +3224,7 @@
         <v>6564</v>
       </c>
     </row>
-    <row r="101" spans="1:6">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>6</v>
       </c>
@@ -3240,7 +3244,7 @@
         <v>6564</v>
       </c>
     </row>
-    <row r="102" spans="1:6">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>6</v>
       </c>
@@ -3260,7 +3264,7 @@
         <v>6565</v>
       </c>
     </row>
-    <row r="103" spans="1:6">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>6</v>
       </c>
@@ -3280,7 +3284,7 @@
         <v>6565</v>
       </c>
     </row>
-    <row r="104" spans="1:6">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>6</v>
       </c>
@@ -3300,7 +3304,7 @@
         <v>6566</v>
       </c>
     </row>
-    <row r="105" spans="1:6">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>6</v>
       </c>
@@ -3320,7 +3324,7 @@
         <v>6566</v>
       </c>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>6</v>
       </c>
@@ -3340,7 +3344,7 @@
         <v>6567</v>
       </c>
     </row>
-    <row r="107" spans="1:6">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>6</v>
       </c>
@@ -3360,7 +3364,7 @@
         <v>6567</v>
       </c>
     </row>
-    <row r="108" spans="1:6">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>6</v>
       </c>
@@ -3380,7 +3384,7 @@
         <v>6568</v>
       </c>
     </row>
-    <row r="109" spans="1:6">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>6</v>
       </c>
@@ -3400,7 +3404,7 @@
         <v>6568</v>
       </c>
     </row>
-    <row r="110" spans="1:6">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>6</v>
       </c>
@@ -3420,7 +3424,7 @@
         <v>6569</v>
       </c>
     </row>
-    <row r="111" spans="1:6">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>6</v>
       </c>
@@ -3440,7 +3444,7 @@
         <v>6569</v>
       </c>
     </row>
-    <row r="112" spans="1:6">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>6</v>
       </c>
@@ -3460,7 +3464,7 @@
         <v>6570</v>
       </c>
     </row>
-    <row r="113" spans="1:6">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>6</v>
       </c>
@@ -3480,7 +3484,7 @@
         <v>6570</v>
       </c>
     </row>
-    <row r="114" spans="1:6">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>6</v>
       </c>
@@ -3500,7 +3504,7 @@
         <v>6571</v>
       </c>
     </row>
-    <row r="115" spans="1:6">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>6</v>
       </c>
@@ -3520,7 +3524,7 @@
         <v>6571</v>
       </c>
     </row>
-    <row r="116" spans="1:6">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>6</v>
       </c>
@@ -3540,7 +3544,7 @@
         <v>6572</v>
       </c>
     </row>
-    <row r="117" spans="1:6">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>6</v>
       </c>
@@ -3560,7 +3564,7 @@
         <v>6572</v>
       </c>
     </row>
-    <row r="118" spans="1:6">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>6</v>
       </c>
@@ -3580,7 +3584,7 @@
         <v>6573</v>
       </c>
     </row>
-    <row r="119" spans="1:6">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>6</v>
       </c>
@@ -3600,7 +3604,7 @@
         <v>6573</v>
       </c>
     </row>
-    <row r="120" spans="1:6">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>6</v>
       </c>
@@ -3620,7 +3624,7 @@
         <v>6574</v>
       </c>
     </row>
-    <row r="121" spans="1:6">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>6</v>
       </c>
@@ -3640,7 +3644,7 @@
         <v>6574</v>
       </c>
     </row>
-    <row r="122" spans="1:6">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>6</v>
       </c>
@@ -3660,7 +3664,7 @@
         <v>6575</v>
       </c>
     </row>
-    <row r="123" spans="1:6">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>6</v>
       </c>
@@ -3680,7 +3684,7 @@
         <v>6575</v>
       </c>
     </row>
-    <row r="124" spans="1:6">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>6</v>
       </c>
@@ -3700,7 +3704,7 @@
         <v>6576</v>
       </c>
     </row>
-    <row r="125" spans="1:6">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>6</v>
       </c>
@@ -3720,7 +3724,7 @@
         <v>6576</v>
       </c>
     </row>
-    <row r="126" spans="1:6">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>6</v>
       </c>
@@ -3740,7 +3744,7 @@
         <v>6577</v>
       </c>
     </row>
-    <row r="127" spans="1:6">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>6</v>
       </c>
@@ -3760,7 +3764,7 @@
         <v>6577</v>
       </c>
     </row>
-    <row r="128" spans="1:6">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>6</v>
       </c>
@@ -3780,7 +3784,7 @@
         <v>6578</v>
       </c>
     </row>
-    <row r="129" spans="1:6">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>6</v>
       </c>
@@ -3800,7 +3804,7 @@
         <v>6578</v>
       </c>
     </row>
-    <row r="130" spans="1:6">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>6</v>
       </c>
@@ -3820,7 +3824,7 @@
         <v>6579</v>
       </c>
     </row>
-    <row r="131" spans="1:6">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>6</v>
       </c>
@@ -3840,7 +3844,7 @@
         <v>6579</v>
       </c>
     </row>
-    <row r="132" spans="1:6">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>6</v>
       </c>
@@ -3860,7 +3864,7 @@
         <v>6580</v>
       </c>
     </row>
-    <row r="133" spans="1:6">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>6</v>
       </c>
@@ -3880,7 +3884,7 @@
         <v>6580</v>
       </c>
     </row>
-    <row r="134" spans="1:6">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>6</v>
       </c>
@@ -3900,7 +3904,7 @@
         <v>6581</v>
       </c>
     </row>
-    <row r="135" spans="1:6">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>6</v>
       </c>
@@ -3920,7 +3924,7 @@
         <v>6581</v>
       </c>
     </row>
-    <row r="136" spans="1:6">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>6</v>
       </c>
@@ -3940,7 +3944,7 @@
         <v>6582</v>
       </c>
     </row>
-    <row r="137" spans="1:6">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>6</v>
       </c>
@@ -3960,7 +3964,7 @@
         <v>6582</v>
       </c>
     </row>
-    <row r="138" spans="1:6">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>6</v>
       </c>
@@ -3980,7 +3984,7 @@
         <v>6583</v>
       </c>
     </row>
-    <row r="139" spans="1:6">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>6</v>
       </c>
@@ -4000,7 +4004,7 @@
         <v>6583</v>
       </c>
     </row>
-    <row r="140" spans="1:6">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>6</v>
       </c>
@@ -4020,7 +4024,7 @@
         <v>6585</v>
       </c>
     </row>
-    <row r="141" spans="1:6">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>6</v>
       </c>
@@ -4040,7 +4044,7 @@
         <v>6585</v>
       </c>
     </row>
-    <row r="142" spans="1:6">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>6</v>
       </c>
@@ -4060,7 +4064,7 @@
         <v>6584</v>
       </c>
     </row>
-    <row r="143" spans="1:6">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>6</v>
       </c>
@@ -4080,7 +4084,7 @@
         <v>6584</v>
       </c>
     </row>
-    <row r="144" spans="1:6">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>6</v>
       </c>
@@ -4100,7 +4104,7 @@
         <v>6586</v>
       </c>
     </row>
-    <row r="145" spans="1:6">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>6</v>
       </c>
@@ -4120,7 +4124,7 @@
         <v>6586</v>
       </c>
     </row>
-    <row r="146" spans="1:6">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>6</v>
       </c>
@@ -4140,7 +4144,7 @@
         <v>6587</v>
       </c>
     </row>
-    <row r="147" spans="1:6">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>6</v>
       </c>
@@ -4160,7 +4164,7 @@
         <v>6587</v>
       </c>
     </row>
-    <row r="148" spans="1:6">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>6</v>
       </c>
@@ -4180,7 +4184,7 @@
         <v>6588</v>
       </c>
     </row>
-    <row r="149" spans="1:6">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>6</v>
       </c>
@@ -4200,7 +4204,7 @@
         <v>6588</v>
       </c>
     </row>
-    <row r="150" spans="1:6">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>6</v>
       </c>
@@ -4220,7 +4224,7 @@
         <v>6589</v>
       </c>
     </row>
-    <row r="151" spans="1:6">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>6</v>
       </c>
@@ -4240,7 +4244,7 @@
         <v>6589</v>
       </c>
     </row>
-    <row r="152" spans="1:6">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>6</v>
       </c>
@@ -4260,7 +4264,7 @@
         <v>6590</v>
       </c>
     </row>
-    <row r="153" spans="1:6">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>6</v>
       </c>
@@ -4280,7 +4284,7 @@
         <v>6590</v>
       </c>
     </row>
-    <row r="154" spans="1:6">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>6</v>
       </c>
@@ -4300,7 +4304,7 @@
         <v>6591</v>
       </c>
     </row>
-    <row r="155" spans="1:6">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>6</v>
       </c>
@@ -4320,7 +4324,7 @@
         <v>6591</v>
       </c>
     </row>
-    <row r="156" spans="1:6">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>6</v>
       </c>
@@ -4340,7 +4344,7 @@
         <v>6592</v>
       </c>
     </row>
-    <row r="157" spans="1:6">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>6</v>
       </c>
@@ -4360,7 +4364,7 @@
         <v>6592</v>
       </c>
     </row>
-    <row r="158" spans="1:6">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>6</v>
       </c>
@@ -4380,7 +4384,7 @@
         <v>6593</v>
       </c>
     </row>
-    <row r="159" spans="1:6">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>6</v>
       </c>
@@ -4400,7 +4404,7 @@
         <v>6593</v>
       </c>
     </row>
-    <row r="160" spans="1:6">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>6</v>
       </c>
@@ -4420,7 +4424,7 @@
         <v>6594</v>
       </c>
     </row>
-    <row r="161" spans="1:6">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>6</v>
       </c>
@@ -4440,7 +4444,7 @@
         <v>6594</v>
       </c>
     </row>
-    <row r="162" spans="1:6">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>6</v>
       </c>
@@ -4460,7 +4464,7 @@
         <v>6595</v>
       </c>
     </row>
-    <row r="163" spans="1:6">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>6</v>
       </c>
@@ -4480,7 +4484,7 @@
         <v>6595</v>
       </c>
     </row>
-    <row r="164" spans="1:6">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>6</v>
       </c>
@@ -4500,7 +4504,7 @@
         <v>6596</v>
       </c>
     </row>
-    <row r="165" spans="1:6">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>6</v>
       </c>
@@ -4520,7 +4524,7 @@
         <v>6596</v>
       </c>
     </row>
-    <row r="166" spans="1:6">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>6</v>
       </c>
@@ -4540,7 +4544,7 @@
         <v>6597</v>
       </c>
     </row>
-    <row r="167" spans="1:6">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>6</v>
       </c>
@@ -4560,7 +4564,7 @@
         <v>6597</v>
       </c>
     </row>
-    <row r="168" spans="1:6">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>6</v>
       </c>
@@ -4580,7 +4584,7 @@
         <v>6598</v>
       </c>
     </row>
-    <row r="169" spans="1:6">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>6</v>
       </c>
@@ -4600,7 +4604,7 @@
         <v>6598</v>
       </c>
     </row>
-    <row r="170" spans="1:6">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>6</v>
       </c>
@@ -4620,7 +4624,7 @@
         <v>6599</v>
       </c>
     </row>
-    <row r="171" spans="1:6">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>6</v>
       </c>
@@ -4640,7 +4644,7 @@
         <v>6599</v>
       </c>
     </row>
-    <row r="172" spans="1:6">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>6</v>
       </c>
@@ -4660,7 +4664,7 @@
         <v>6600</v>
       </c>
     </row>
-    <row r="173" spans="1:6">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>6</v>
       </c>
@@ -4680,7 +4684,7 @@
         <v>6600</v>
       </c>
     </row>
-    <row r="174" spans="1:6">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>6</v>
       </c>
@@ -4700,7 +4704,7 @@
         <v>6601</v>
       </c>
     </row>
-    <row r="175" spans="1:6">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>6</v>
       </c>
@@ -4720,7 +4724,7 @@
         <v>6601</v>
       </c>
     </row>
-    <row r="176" spans="1:6">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>6</v>
       </c>
@@ -4740,7 +4744,7 @@
         <v>6602</v>
       </c>
     </row>
-    <row r="177" spans="1:6">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>6</v>
       </c>
@@ -4760,7 +4764,7 @@
         <v>6602</v>
       </c>
     </row>
-    <row r="178" spans="1:6">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>6</v>
       </c>
@@ -4780,7 +4784,7 @@
         <v>6603</v>
       </c>
     </row>
-    <row r="179" spans="1:6">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>6</v>
       </c>
@@ -4800,7 +4804,7 @@
         <v>6603</v>
       </c>
     </row>
-    <row r="180" spans="1:6">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>6</v>
       </c>
@@ -4820,7 +4824,7 @@
         <v>6604</v>
       </c>
     </row>
-    <row r="181" spans="1:6">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>6</v>
       </c>
@@ -4840,7 +4844,7 @@
         <v>6604</v>
       </c>
     </row>
-    <row r="182" spans="1:6">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>6</v>
       </c>
@@ -4860,7 +4864,7 @@
         <v>6605</v>
       </c>
     </row>
-    <row r="183" spans="1:6">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>6</v>
       </c>
@@ -4880,7 +4884,7 @@
         <v>6605</v>
       </c>
     </row>
-    <row r="184" spans="1:6">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>6</v>
       </c>
@@ -4900,7 +4904,7 @@
         <v>6606</v>
       </c>
     </row>
-    <row r="185" spans="1:6">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>6</v>
       </c>
@@ -4920,7 +4924,7 @@
         <v>6606</v>
       </c>
     </row>
-    <row r="186" spans="1:6">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>6</v>
       </c>
@@ -4940,7 +4944,7 @@
         <v>6607</v>
       </c>
     </row>
-    <row r="187" spans="1:6">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>6</v>
       </c>
@@ -4960,7 +4964,7 @@
         <v>6607</v>
       </c>
     </row>
-    <row r="188" spans="1:6">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>6</v>
       </c>
@@ -4980,7 +4984,7 @@
         <v>6608</v>
       </c>
     </row>
-    <row r="189" spans="1:6">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>6</v>
       </c>
@@ -5000,7 +5004,7 @@
         <v>6608</v>
       </c>
     </row>
-    <row r="190" spans="1:6">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>6</v>
       </c>
@@ -5020,7 +5024,7 @@
         <v>6609</v>
       </c>
     </row>
-    <row r="191" spans="1:6">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>6</v>
       </c>
@@ -5040,7 +5044,7 @@
         <v>6609</v>
       </c>
     </row>
-    <row r="192" spans="1:6">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>6</v>
       </c>
@@ -5060,7 +5064,7 @@
         <v>6610</v>
       </c>
     </row>
-    <row r="193" spans="1:6">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>6</v>
       </c>
@@ -5080,7 +5084,7 @@
         <v>6610</v>
       </c>
     </row>
-    <row r="194" spans="1:6">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>6</v>
       </c>
@@ -5100,7 +5104,7 @@
         <v>6611</v>
       </c>
     </row>
-    <row r="195" spans="1:6">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>6</v>
       </c>
@@ -5120,7 +5124,7 @@
         <v>6611</v>
       </c>
     </row>
-    <row r="196" spans="1:6">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>6</v>
       </c>
@@ -5140,7 +5144,7 @@
         <v>6612</v>
       </c>
     </row>
-    <row r="197" spans="1:6">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>6</v>
       </c>
@@ -5160,7 +5164,7 @@
         <v>6612</v>
       </c>
     </row>
-    <row r="198" spans="1:6">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>6</v>
       </c>
@@ -5180,7 +5184,7 @@
         <v>6613</v>
       </c>
     </row>
-    <row r="199" spans="1:6">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>6</v>
       </c>
@@ -5200,7 +5204,7 @@
         <v>6613</v>
       </c>
     </row>
-    <row r="200" spans="1:6">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>6</v>
       </c>
@@ -5220,7 +5224,7 @@
         <v>6614</v>
       </c>
     </row>
-    <row r="201" spans="1:6">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>6</v>
       </c>
@@ -5240,7 +5244,7 @@
         <v>6614</v>
       </c>
     </row>
-    <row r="202" spans="1:6">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>6</v>
       </c>
@@ -5260,7 +5264,7 @@
         <v>6615</v>
       </c>
     </row>
-    <row r="203" spans="1:6">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>6</v>
       </c>
@@ -5280,7 +5284,7 @@
         <v>6615</v>
       </c>
     </row>
-    <row r="204" spans="1:6">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>6</v>
       </c>
@@ -5300,7 +5304,7 @@
         <v>6616</v>
       </c>
     </row>
-    <row r="205" spans="1:6">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>6</v>
       </c>
@@ -5320,7 +5324,7 @@
         <v>6616</v>
       </c>
     </row>
-    <row r="206" spans="1:6">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>6</v>
       </c>
@@ -5340,7 +5344,7 @@
         <v>6617</v>
       </c>
     </row>
-    <row r="207" spans="1:6">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>6</v>
       </c>
@@ -5360,7 +5364,7 @@
         <v>6617</v>
       </c>
     </row>
-    <row r="208" spans="1:6">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>6</v>
       </c>
@@ -5380,7 +5384,7 @@
         <v>6618</v>
       </c>
     </row>
-    <row r="209" spans="1:6">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>6</v>
       </c>
@@ -5400,7 +5404,7 @@
         <v>6618</v>
       </c>
     </row>
-    <row r="210" spans="1:6">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>6</v>
       </c>
@@ -5420,7 +5424,7 @@
         <v>6619</v>
       </c>
     </row>
-    <row r="211" spans="1:6">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>6</v>
       </c>
@@ -5440,7 +5444,7 @@
         <v>6619</v>
       </c>
     </row>
-    <row r="212" spans="1:6">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>6</v>
       </c>
@@ -5460,7 +5464,7 @@
         <v>6620</v>
       </c>
     </row>
-    <row r="213" spans="1:6">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>6</v>
       </c>
@@ -5480,7 +5484,7 @@
         <v>6620</v>
       </c>
     </row>
-    <row r="214" spans="1:6">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>6</v>
       </c>
@@ -5500,7 +5504,7 @@
         <v>6621</v>
       </c>
     </row>
-    <row r="215" spans="1:6">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>6</v>
       </c>
@@ -5520,7 +5524,7 @@
         <v>6621</v>
       </c>
     </row>
-    <row r="216" spans="1:6">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>6</v>
       </c>
@@ -5540,7 +5544,7 @@
         <v>6622</v>
       </c>
     </row>
-    <row r="217" spans="1:6">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>6</v>
       </c>
@@ -5560,7 +5564,7 @@
         <v>6622</v>
       </c>
     </row>
-    <row r="218" spans="1:6">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>6</v>
       </c>
@@ -5580,7 +5584,7 @@
         <v>6623</v>
       </c>
     </row>
-    <row r="219" spans="1:6">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>6</v>
       </c>
@@ -5600,7 +5604,7 @@
         <v>6623</v>
       </c>
     </row>
-    <row r="220" spans="1:6">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>6</v>
       </c>
@@ -5620,7 +5624,7 @@
         <v>6624</v>
       </c>
     </row>
-    <row r="221" spans="1:6">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>6</v>
       </c>
@@ -5640,7 +5644,7 @@
         <v>6624</v>
       </c>
     </row>
-    <row r="222" spans="1:6">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>6</v>
       </c>
@@ -5660,7 +5664,7 @@
         <v>6625</v>
       </c>
     </row>
-    <row r="223" spans="1:6">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>6</v>
       </c>
@@ -5680,7 +5684,7 @@
         <v>6625</v>
       </c>
     </row>
-    <row r="224" spans="1:6">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>6</v>
       </c>
@@ -5700,7 +5704,7 @@
         <v>6626</v>
       </c>
     </row>
-    <row r="225" spans="1:6">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>6</v>
       </c>
@@ -5720,7 +5724,7 @@
         <v>6626</v>
       </c>
     </row>
-    <row r="226" spans="1:6">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>6</v>
       </c>
@@ -5740,7 +5744,7 @@
         <v>6627</v>
       </c>
     </row>
-    <row r="227" spans="1:6">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>6</v>
       </c>
@@ -5760,7 +5764,7 @@
         <v>6627</v>
       </c>
     </row>
-    <row r="228" spans="1:6">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>6</v>
       </c>
@@ -5780,7 +5784,7 @@
         <v>6628</v>
       </c>
     </row>
-    <row r="229" spans="1:6">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>6</v>
       </c>
@@ -5800,7 +5804,7 @@
         <v>6628</v>
       </c>
     </row>
-    <row r="230" spans="1:6">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>6</v>
       </c>
@@ -5820,7 +5824,7 @@
         <v>6629</v>
       </c>
     </row>
-    <row r="231" spans="1:6">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>6</v>
       </c>
@@ -5840,7 +5844,7 @@
         <v>6629</v>
       </c>
     </row>
-    <row r="232" spans="1:6">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>6</v>
       </c>
@@ -5860,7 +5864,7 @@
         <v>6630</v>
       </c>
     </row>
-    <row r="233" spans="1:6">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>6</v>
       </c>
@@ -5880,7 +5884,7 @@
         <v>6630</v>
       </c>
     </row>
-    <row r="234" spans="1:6">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>6</v>
       </c>
@@ -5900,7 +5904,7 @@
         <v>6631</v>
       </c>
     </row>
-    <row r="235" spans="1:6">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>6</v>
       </c>
@@ -5920,7 +5924,7 @@
         <v>6631</v>
       </c>
     </row>
-    <row r="236" spans="1:6">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>6</v>
       </c>
@@ -5940,7 +5944,7 @@
         <v>6632</v>
       </c>
     </row>
-    <row r="237" spans="1:6">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>6</v>
       </c>
@@ -5960,7 +5964,7 @@
         <v>6632</v>
       </c>
     </row>
-    <row r="238" spans="1:6">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>6</v>
       </c>
@@ -5980,7 +5984,7 @@
         <v>6633</v>
       </c>
     </row>
-    <row r="239" spans="1:6">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>6</v>
       </c>
@@ -6000,7 +6004,7 @@
         <v>6633</v>
       </c>
     </row>
-    <row r="240" spans="1:6">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>6</v>
       </c>
@@ -6020,7 +6024,7 @@
         <v>6634</v>
       </c>
     </row>
-    <row r="241" spans="1:6">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>6</v>
       </c>
@@ -6040,7 +6044,7 @@
         <v>6634</v>
       </c>
     </row>
-    <row r="242" spans="1:6">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>6</v>
       </c>
@@ -6060,7 +6064,7 @@
         <v>6635</v>
       </c>
     </row>
-    <row r="243" spans="1:6">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>6</v>
       </c>
@@ -6080,7 +6084,7 @@
         <v>6635</v>
       </c>
     </row>
-    <row r="244" spans="1:6">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>6</v>
       </c>
@@ -6100,7 +6104,7 @@
         <v>6636</v>
       </c>
     </row>
-    <row r="245" spans="1:6">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>6</v>
       </c>
@@ -6120,7 +6124,7 @@
         <v>6636</v>
       </c>
     </row>
-    <row r="246" spans="1:6">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>6</v>
       </c>
@@ -6140,7 +6144,7 @@
         <v>6637</v>
       </c>
     </row>
-    <row r="247" spans="1:6">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>6</v>
       </c>
@@ -6160,7 +6164,7 @@
         <v>6637</v>
       </c>
     </row>
-    <row r="248" spans="1:6">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>6</v>
       </c>
@@ -6180,7 +6184,7 @@
         <v>6638</v>
       </c>
     </row>
-    <row r="249" spans="1:6">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>6</v>
       </c>
@@ -6200,7 +6204,7 @@
         <v>6638</v>
       </c>
     </row>
-    <row r="250" spans="1:6">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>6</v>
       </c>
@@ -6220,7 +6224,7 @@
         <v>6639</v>
       </c>
     </row>
-    <row r="251" spans="1:6">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>6</v>
       </c>
@@ -6240,7 +6244,7 @@
         <v>6639</v>
       </c>
     </row>
-    <row r="252" spans="1:6">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>6</v>
       </c>
@@ -6260,7 +6264,7 @@
         <v>6640</v>
       </c>
     </row>
-    <row r="253" spans="1:6">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>6</v>
       </c>
@@ -6280,7 +6284,7 @@
         <v>6640</v>
       </c>
     </row>
-    <row r="254" spans="1:6">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>6</v>
       </c>
@@ -6300,7 +6304,7 @@
         <v>6641</v>
       </c>
     </row>
-    <row r="255" spans="1:6">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>6</v>
       </c>
@@ -6320,7 +6324,7 @@
         <v>6641</v>
       </c>
     </row>
-    <row r="256" spans="1:6">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>6</v>
       </c>
@@ -6340,7 +6344,7 @@
         <v>6642</v>
       </c>
     </row>
-    <row r="257" spans="1:6">
+    <row r="257" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>6</v>
       </c>
@@ -6360,7 +6364,7 @@
         <v>6642</v>
       </c>
     </row>
-    <row r="258" spans="1:6">
+    <row r="258" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>6</v>
       </c>
@@ -6380,7 +6384,7 @@
         <v>6643</v>
       </c>
     </row>
-    <row r="259" spans="1:6">
+    <row r="259" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>6</v>
       </c>
@@ -6400,7 +6404,7 @@
         <v>6643</v>
       </c>
     </row>
-    <row r="260" spans="1:6">
+    <row r="260" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>6</v>
       </c>
@@ -6420,7 +6424,7 @@
         <v>6644</v>
       </c>
     </row>
-    <row r="261" spans="1:6">
+    <row r="261" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>6</v>
       </c>
@@ -6440,7 +6444,7 @@
         <v>6644</v>
       </c>
     </row>
-    <row r="262" spans="1:6">
+    <row r="262" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>6</v>
       </c>
@@ -6460,7 +6464,7 @@
         <v>6645</v>
       </c>
     </row>
-    <row r="263" spans="1:6">
+    <row r="263" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>6</v>
       </c>
@@ -6480,7 +6484,7 @@
         <v>6645</v>
       </c>
     </row>
-    <row r="264" spans="1:6">
+    <row r="264" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>6</v>
       </c>
@@ -6500,7 +6504,7 @@
         <v>6646</v>
       </c>
     </row>
-    <row r="265" spans="1:6">
+    <row r="265" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>6</v>
       </c>
@@ -6520,7 +6524,7 @@
         <v>6646</v>
       </c>
     </row>
-    <row r="266" spans="1:6">
+    <row r="266" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>6</v>
       </c>
@@ -6540,7 +6544,7 @@
         <v>6647</v>
       </c>
     </row>
-    <row r="267" spans="1:6">
+    <row r="267" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>6</v>
       </c>
@@ -6560,7 +6564,7 @@
         <v>6647</v>
       </c>
     </row>
-    <row r="268" spans="1:6">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>6</v>
       </c>
@@ -6580,7 +6584,7 @@
         <v>6648</v>
       </c>
     </row>
-    <row r="269" spans="1:6">
+    <row r="269" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>6</v>
       </c>
@@ -6600,7 +6604,7 @@
         <v>6648</v>
       </c>
     </row>
-    <row r="270" spans="1:6">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>6</v>
       </c>
@@ -6620,7 +6624,7 @@
         <v>6649</v>
       </c>
     </row>
-    <row r="271" spans="1:6">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>6</v>
       </c>
@@ -6640,7 +6644,7 @@
         <v>6649</v>
       </c>
     </row>
-    <row r="272" spans="1:6">
+    <row r="272" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>6</v>
       </c>
@@ -6660,7 +6664,7 @@
         <v>6650</v>
       </c>
     </row>
-    <row r="273" spans="1:6">
+    <row r="273" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>6</v>
       </c>
@@ -6680,7 +6684,7 @@
         <v>6650</v>
       </c>
     </row>
-    <row r="274" spans="1:6">
+    <row r="274" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>6</v>
       </c>
@@ -6700,7 +6704,7 @@
         <v>6651</v>
       </c>
     </row>
-    <row r="275" spans="1:6">
+    <row r="275" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>6</v>
       </c>
@@ -6720,7 +6724,7 @@
         <v>6651</v>
       </c>
     </row>
-    <row r="276" spans="1:6">
+    <row r="276" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>6</v>
       </c>
@@ -6740,7 +6744,7 @@
         <v>6652</v>
       </c>
     </row>
-    <row r="277" spans="1:6">
+    <row r="277" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>6</v>
       </c>
@@ -6760,7 +6764,7 @@
         <v>6652</v>
       </c>
     </row>
-    <row r="278" spans="1:6">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>6</v>
       </c>
@@ -6780,7 +6784,7 @@
         <v>6656</v>
       </c>
     </row>
-    <row r="279" spans="1:6">
+    <row r="279" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>6</v>
       </c>
@@ -6800,7 +6804,7 @@
         <v>6656</v>
       </c>
     </row>
-    <row r="280" spans="1:6">
+    <row r="280" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>6</v>
       </c>
@@ -6820,7 +6824,7 @@
         <v>6653</v>
       </c>
     </row>
-    <row r="281" spans="1:6">
+    <row r="281" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>6</v>
       </c>
@@ -6840,7 +6844,7 @@
         <v>6653</v>
       </c>
     </row>
-    <row r="282" spans="1:6">
+    <row r="282" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>6</v>
       </c>
@@ -6860,7 +6864,7 @@
         <v>6654</v>
       </c>
     </row>
-    <row r="283" spans="1:6">
+    <row r="283" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>6</v>
       </c>
@@ -6880,7 +6884,7 @@
         <v>6654</v>
       </c>
     </row>
-    <row r="284" spans="1:6">
+    <row r="284" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>6</v>
       </c>
@@ -6900,7 +6904,7 @@
         <v>6655</v>
       </c>
     </row>
-    <row r="285" spans="1:6">
+    <row r="285" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>6</v>
       </c>
@@ -6920,7 +6924,7 @@
         <v>6655</v>
       </c>
     </row>
-    <row r="286" spans="1:6">
+    <row r="286" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>6</v>
       </c>
@@ -6940,7 +6944,7 @@
         <v>6657</v>
       </c>
     </row>
-    <row r="287" spans="1:6">
+    <row r="287" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>6</v>
       </c>
@@ -6960,7 +6964,7 @@
         <v>6657</v>
       </c>
     </row>
-    <row r="288" spans="1:6">
+    <row r="288" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>6</v>
       </c>
@@ -6980,7 +6984,7 @@
         <v>6658</v>
       </c>
     </row>
-    <row r="289" spans="1:6">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>6</v>
       </c>
@@ -7000,7 +7004,7 @@
         <v>6658</v>
       </c>
     </row>
-    <row r="290" spans="1:6">
+    <row r="290" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>6</v>
       </c>
@@ -7020,7 +7024,7 @@
         <v>6659</v>
       </c>
     </row>
-    <row r="291" spans="1:6">
+    <row r="291" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>6</v>
       </c>
@@ -7040,7 +7044,7 @@
         <v>6659</v>
       </c>
     </row>
-    <row r="292" spans="1:6">
+    <row r="292" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>6</v>
       </c>
@@ -7060,7 +7064,7 @@
         <v>6660</v>
       </c>
     </row>
-    <row r="293" spans="1:6">
+    <row r="293" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>6</v>
       </c>
@@ -7080,7 +7084,7 @@
         <v>6660</v>
       </c>
     </row>
-    <row r="294" spans="1:6">
+    <row r="294" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>6</v>
       </c>
@@ -7100,7 +7104,7 @@
         <v>6661</v>
       </c>
     </row>
-    <row r="295" spans="1:6">
+    <row r="295" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>6</v>
       </c>
@@ -7120,7 +7124,7 @@
         <v>6661</v>
       </c>
     </row>
-    <row r="296" spans="1:6">
+    <row r="296" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>6</v>
       </c>
@@ -7140,7 +7144,7 @@
         <v>6662</v>
       </c>
     </row>
-    <row r="297" spans="1:6">
+    <row r="297" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>6</v>
       </c>
@@ -7160,7 +7164,7 @@
         <v>6662</v>
       </c>
     </row>
-    <row r="298" spans="1:6">
+    <row r="298" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>6</v>
       </c>
@@ -7180,7 +7184,7 @@
         <v>6663</v>
       </c>
     </row>
-    <row r="299" spans="1:6">
+    <row r="299" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>6</v>
       </c>
@@ -7200,7 +7204,7 @@
         <v>6663</v>
       </c>
     </row>
-    <row r="300" spans="1:6">
+    <row r="300" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>6</v>
       </c>
@@ -7220,7 +7224,7 @@
         <v>6664</v>
       </c>
     </row>
-    <row r="301" spans="1:6">
+    <row r="301" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>6</v>
       </c>
@@ -7240,7 +7244,7 @@
         <v>6664</v>
       </c>
     </row>
-    <row r="302" spans="1:6">
+    <row r="302" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>6</v>
       </c>
@@ -7260,7 +7264,7 @@
         <v>6665</v>
       </c>
     </row>
-    <row r="303" spans="1:6">
+    <row r="303" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>6</v>
       </c>
@@ -7280,7 +7284,7 @@
         <v>6665</v>
       </c>
     </row>
-    <row r="304" spans="1:6">
+    <row r="304" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>6</v>
       </c>
@@ -7300,7 +7304,7 @@
         <v>6666</v>
       </c>
     </row>
-    <row r="305" spans="1:6">
+    <row r="305" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>6</v>
       </c>
@@ -7320,7 +7324,7 @@
         <v>6666</v>
       </c>
     </row>
-    <row r="306" spans="1:6">
+    <row r="306" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>6</v>
       </c>
@@ -7340,7 +7344,7 @@
         <v>6667</v>
       </c>
     </row>
-    <row r="307" spans="1:6">
+    <row r="307" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>6</v>
       </c>
@@ -7360,7 +7364,7 @@
         <v>6667</v>
       </c>
     </row>
-    <row r="308" spans="1:6">
+    <row r="308" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>6</v>
       </c>
@@ -7380,7 +7384,7 @@
         <v>6671</v>
       </c>
     </row>
-    <row r="309" spans="1:6">
+    <row r="309" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>6</v>
       </c>
@@ -7400,7 +7404,7 @@
         <v>6671</v>
       </c>
     </row>
-    <row r="310" spans="1:6">
+    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>6</v>
       </c>
@@ -7420,7 +7424,7 @@
         <v>6672</v>
       </c>
     </row>
-    <row r="311" spans="1:6">
+    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>6</v>
       </c>
@@ -7440,7 +7444,7 @@
         <v>6672</v>
       </c>
     </row>
-    <row r="312" spans="1:6">
+    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>6</v>
       </c>
@@ -7460,7 +7464,7 @@
         <v>6673</v>
       </c>
     </row>
-    <row r="313" spans="1:6">
+    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>6</v>
       </c>
@@ -7480,7 +7484,7 @@
         <v>6673</v>
       </c>
     </row>
-    <row r="314" spans="1:6">
+    <row r="314" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>6</v>
       </c>
@@ -7500,7 +7504,7 @@
         <v>6674</v>
       </c>
     </row>
-    <row r="315" spans="1:6">
+    <row r="315" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>6</v>
       </c>
@@ -7520,7 +7524,7 @@
         <v>6674</v>
       </c>
     </row>
-    <row r="316" spans="1:6">
+    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>6</v>
       </c>
@@ -7540,7 +7544,7 @@
         <v>6675</v>
       </c>
     </row>
-    <row r="317" spans="1:6">
+    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>6</v>
       </c>
@@ -7560,7 +7564,7 @@
         <v>6675</v>
       </c>
     </row>
-    <row r="318" spans="1:6">
+    <row r="318" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>6</v>
       </c>
@@ -7580,7 +7584,7 @@
         <v>6676</v>
       </c>
     </row>
-    <row r="319" spans="1:6">
+    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>6</v>
       </c>
@@ -7600,7 +7604,7 @@
         <v>6676</v>
       </c>
     </row>
-    <row r="320" spans="1:6">
+    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>6</v>
       </c>
@@ -7620,7 +7624,7 @@
         <v>6668</v>
       </c>
     </row>
-    <row r="321" spans="1:6">
+    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>6</v>
       </c>
@@ -7640,7 +7644,7 @@
         <v>6668</v>
       </c>
     </row>
-    <row r="322" spans="1:6">
+    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>6</v>
       </c>
@@ -7660,7 +7664,7 @@
         <v>6669</v>
       </c>
     </row>
-    <row r="323" spans="1:6">
+    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>6</v>
       </c>
@@ -7680,7 +7684,7 @@
         <v>6669</v>
       </c>
     </row>
-    <row r="324" spans="1:6">
+    <row r="324" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
         <v>6</v>
       </c>
@@ -7700,7 +7704,7 @@
         <v>6670</v>
       </c>
     </row>
-    <row r="325" spans="1:6">
+    <row r="325" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>6</v>
       </c>
@@ -7720,7 +7724,7 @@
         <v>6670</v>
       </c>
     </row>
-    <row r="326" spans="1:6">
+    <row r="326" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>6</v>
       </c>
@@ -7740,7 +7744,7 @@
         <v>6677</v>
       </c>
     </row>
-    <row r="327" spans="1:6">
+    <row r="327" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
         <v>6</v>
       </c>
@@ -7760,7 +7764,7 @@
         <v>6677</v>
       </c>
     </row>
-    <row r="328" spans="1:6">
+    <row r="328" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
         <v>6</v>
       </c>
@@ -7780,7 +7784,7 @@
         <v>6678</v>
       </c>
     </row>
-    <row r="329" spans="1:6">
+    <row r="329" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
         <v>6</v>
       </c>
@@ -7800,7 +7804,7 @@
         <v>6678</v>
       </c>
     </row>
-    <row r="330" spans="1:6">
+    <row r="330" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
         <v>6</v>
       </c>
@@ -7820,7 +7824,7 @@
         <v>6679</v>
       </c>
     </row>
-    <row r="331" spans="1:6">
+    <row r="331" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
         <v>6</v>
       </c>
@@ -7840,7 +7844,7 @@
         <v>6679</v>
       </c>
     </row>
-    <row r="332" spans="1:6">
+    <row r="332" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
         <v>6</v>
       </c>
@@ -7860,7 +7864,7 @@
         <v>6680</v>
       </c>
     </row>
-    <row r="333" spans="1:6">
+    <row r="333" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
         <v>6</v>
       </c>
@@ -7880,7 +7884,7 @@
         <v>6680</v>
       </c>
     </row>
-    <row r="334" spans="1:6">
+    <row r="334" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
         <v>6</v>
       </c>
@@ -7900,7 +7904,7 @@
         <v>6681</v>
       </c>
     </row>
-    <row r="335" spans="1:6">
+    <row r="335" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
         <v>6</v>
       </c>
@@ -7920,7 +7924,7 @@
         <v>6681</v>
       </c>
     </row>
-    <row r="336" spans="1:6">
+    <row r="336" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
         <v>6</v>
       </c>
@@ -7940,7 +7944,7 @@
         <v>6682</v>
       </c>
     </row>
-    <row r="337" spans="1:6">
+    <row r="337" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>6</v>
       </c>
@@ -7960,7 +7964,7 @@
         <v>6682</v>
       </c>
     </row>
-    <row r="338" spans="1:6">
+    <row r="338" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>6</v>
       </c>
@@ -7980,7 +7984,7 @@
         <v>6683</v>
       </c>
     </row>
-    <row r="339" spans="1:6">
+    <row r="339" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>6</v>
       </c>
@@ -8000,7 +8004,7 @@
         <v>6683</v>
       </c>
     </row>
-    <row r="340" spans="1:6">
+    <row r="340" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>6</v>
       </c>
@@ -8020,7 +8024,7 @@
         <v>6684</v>
       </c>
     </row>
-    <row r="341" spans="1:6">
+    <row r="341" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>6</v>
       </c>
@@ -8040,7 +8044,7 @@
         <v>6684</v>
       </c>
     </row>
-    <row r="342" spans="1:6">
+    <row r="342" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
         <v>6</v>
       </c>
@@ -8060,7 +8064,7 @@
         <v>6685</v>
       </c>
     </row>
-    <row r="343" spans="1:6">
+    <row r="343" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
         <v>6</v>
       </c>
@@ -8080,7 +8084,7 @@
         <v>6685</v>
       </c>
     </row>
-    <row r="344" spans="1:6">
+    <row r="344" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
         <v>6</v>
       </c>
@@ -8100,7 +8104,7 @@
         <v>6686</v>
       </c>
     </row>
-    <row r="345" spans="1:6">
+    <row r="345" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
         <v>6</v>
       </c>
@@ -8120,7 +8124,7 @@
         <v>6686</v>
       </c>
     </row>
-    <row r="346" spans="1:6">
+    <row r="346" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
         <v>6</v>
       </c>
@@ -8140,7 +8144,7 @@
         <v>6687</v>
       </c>
     </row>
-    <row r="347" spans="1:6">
+    <row r="347" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
         <v>6</v>
       </c>
@@ -8160,7 +8164,7 @@
         <v>6687</v>
       </c>
     </row>
-    <row r="348" spans="1:6">
+    <row r="348" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
         <v>6</v>
       </c>
@@ -8180,7 +8184,7 @@
         <v>6688</v>
       </c>
     </row>
-    <row r="349" spans="1:6">
+    <row r="349" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
         <v>6</v>
       </c>
@@ -8200,7 +8204,7 @@
         <v>6688</v>
       </c>
     </row>
-    <row r="350" spans="1:6">
+    <row r="350" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
         <v>6</v>
       </c>
@@ -8220,7 +8224,7 @@
         <v>6689</v>
       </c>
     </row>
-    <row r="351" spans="1:6">
+    <row r="351" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
         <v>6</v>
       </c>
@@ -8240,7 +8244,7 @@
         <v>6689</v>
       </c>
     </row>
-    <row r="352" spans="1:6">
+    <row r="352" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
         <v>6</v>
       </c>
@@ -8260,7 +8264,7 @@
         <v>6690</v>
       </c>
     </row>
-    <row r="353" spans="1:6">
+    <row r="353" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
         <v>6</v>
       </c>
@@ -8280,7 +8284,7 @@
         <v>6690</v>
       </c>
     </row>
-    <row r="354" spans="1:6">
+    <row r="354" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
         <v>6</v>
       </c>
@@ -8300,7 +8304,7 @@
         <v>6691</v>
       </c>
     </row>
-    <row r="355" spans="1:6">
+    <row r="355" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
         <v>6</v>
       </c>
@@ -8320,7 +8324,7 @@
         <v>6691</v>
       </c>
     </row>
-    <row r="356" spans="1:6">
+    <row r="356" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
         <v>6</v>
       </c>
@@ -8340,7 +8344,7 @@
         <v>6692</v>
       </c>
     </row>
-    <row r="357" spans="1:6">
+    <row r="357" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
         <v>6</v>
       </c>
@@ -8360,7 +8364,7 @@
         <v>6692</v>
       </c>
     </row>
-    <row r="358" spans="1:6">
+    <row r="358" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
         <v>6</v>
       </c>
@@ -8380,7 +8384,7 @@
         <v>6693</v>
       </c>
     </row>
-    <row r="359" spans="1:6">
+    <row r="359" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
         <v>6</v>
       </c>
@@ -8400,7 +8404,7 @@
         <v>6693</v>
       </c>
     </row>
-    <row r="360" spans="1:6">
+    <row r="360" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
         <v>6</v>
       </c>
@@ -8420,7 +8424,7 @@
         <v>6694</v>
       </c>
     </row>
-    <row r="361" spans="1:6">
+    <row r="361" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
         <v>6</v>
       </c>
@@ -8440,7 +8444,7 @@
         <v>6694</v>
       </c>
     </row>
-    <row r="362" spans="1:6">
+    <row r="362" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
         <v>6</v>
       </c>
@@ -8460,7 +8464,7 @@
         <v>6695</v>
       </c>
     </row>
-    <row r="363" spans="1:6">
+    <row r="363" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
         <v>6</v>
       </c>
@@ -8480,7 +8484,7 @@
         <v>6695</v>
       </c>
     </row>
-    <row r="364" spans="1:6">
+    <row r="364" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
         <v>6</v>
       </c>
@@ -8500,7 +8504,7 @@
         <v>6696</v>
       </c>
     </row>
-    <row r="365" spans="1:6">
+    <row r="365" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
         <v>6</v>
       </c>
@@ -8520,7 +8524,7 @@
         <v>6696</v>
       </c>
     </row>
-    <row r="366" spans="1:6">
+    <row r="366" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
         <v>6</v>
       </c>
@@ -8540,7 +8544,7 @@
         <v>6697</v>
       </c>
     </row>
-    <row r="367" spans="1:6">
+    <row r="367" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
         <v>6</v>
       </c>
@@ -8560,7 +8564,7 @@
         <v>6697</v>
       </c>
     </row>
-    <row r="368" spans="1:6">
+    <row r="368" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
         <v>6</v>
       </c>
@@ -8580,7 +8584,7 @@
         <v>6698</v>
       </c>
     </row>
-    <row r="369" spans="1:6">
+    <row r="369" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
         <v>6</v>
       </c>
@@ -8600,7 +8604,7 @@
         <v>6698</v>
       </c>
     </row>
-    <row r="370" spans="1:6">
+    <row r="370" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
         <v>6</v>
       </c>
@@ -8620,7 +8624,7 @@
         <v>6699</v>
       </c>
     </row>
-    <row r="371" spans="1:6">
+    <row r="371" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
         <v>6</v>
       </c>
@@ -8640,7 +8644,7 @@
         <v>6699</v>
       </c>
     </row>
-    <row r="372" spans="1:6">
+    <row r="372" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
         <v>6</v>
       </c>
@@ -8660,7 +8664,7 @@
         <v>6700</v>
       </c>
     </row>
-    <row r="373" spans="1:6">
+    <row r="373" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
         <v>6</v>
       </c>
@@ -8680,7 +8684,7 @@
         <v>6700</v>
       </c>
     </row>
-    <row r="374" spans="1:6">
+    <row r="374" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
         <v>6</v>
       </c>
@@ -8700,7 +8704,7 @@
         <v>6701</v>
       </c>
     </row>
-    <row r="375" spans="1:6">
+    <row r="375" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
         <v>6</v>
       </c>
@@ -8720,7 +8724,7 @@
         <v>6701</v>
       </c>
     </row>
-    <row r="376" spans="1:6">
+    <row r="376" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
         <v>6</v>
       </c>
@@ -8740,7 +8744,7 @@
         <v>6702</v>
       </c>
     </row>
-    <row r="377" spans="1:6">
+    <row r="377" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
         <v>6</v>
       </c>
@@ -8760,7 +8764,7 @@
         <v>6702</v>
       </c>
     </row>
-    <row r="378" spans="1:6">
+    <row r="378" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
         <v>6</v>
       </c>
@@ -8780,7 +8784,7 @@
         <v>6703</v>
       </c>
     </row>
-    <row r="379" spans="1:6">
+    <row r="379" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
         <v>6</v>
       </c>
@@ -8800,7 +8804,7 @@
         <v>6703</v>
       </c>
     </row>
-    <row r="380" spans="1:6">
+    <row r="380" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
         <v>6</v>
       </c>
@@ -8820,7 +8824,7 @@
         <v>6704</v>
       </c>
     </row>
-    <row r="381" spans="1:6">
+    <row r="381" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
         <v>6</v>
       </c>
@@ -8840,7 +8844,7 @@
         <v>6704</v>
       </c>
     </row>
-    <row r="382" spans="1:6">
+    <row r="382" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
         <v>6</v>
       </c>
@@ -8860,7 +8864,7 @@
         <v>6705</v>
       </c>
     </row>
-    <row r="383" spans="1:6">
+    <row r="383" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
         <v>6</v>
       </c>
@@ -8880,7 +8884,7 @@
         <v>6705</v>
       </c>
     </row>
-    <row r="384" spans="1:6">
+    <row r="384" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
         <v>6</v>
       </c>
@@ -8900,7 +8904,7 @@
         <v>6706</v>
       </c>
     </row>
-    <row r="385" spans="1:6">
+    <row r="385" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
         <v>6</v>
       </c>
@@ -8920,7 +8924,7 @@
         <v>6706</v>
       </c>
     </row>
-    <row r="386" spans="1:6">
+    <row r="386" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
         <v>6</v>
       </c>
@@ -8940,7 +8944,7 @@
         <v>6707</v>
       </c>
     </row>
-    <row r="387" spans="1:6">
+    <row r="387" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
         <v>6</v>
       </c>
@@ -8960,7 +8964,7 @@
         <v>6707</v>
       </c>
     </row>
-    <row r="388" spans="1:6">
+    <row r="388" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
         <v>6</v>
       </c>
@@ -8980,7 +8984,7 @@
         <v>6708</v>
       </c>
     </row>
-    <row r="389" spans="1:6">
+    <row r="389" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
         <v>6</v>
       </c>
@@ -9000,7 +9004,7 @@
         <v>6708</v>
       </c>
     </row>
-    <row r="390" spans="1:6">
+    <row r="390" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
         <v>6</v>
       </c>
@@ -9020,7 +9024,7 @@
         <v>6709</v>
       </c>
     </row>
-    <row r="391" spans="1:6">
+    <row r="391" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
         <v>6</v>
       </c>
@@ -9040,7 +9044,7 @@
         <v>6709</v>
       </c>
     </row>
-    <row r="392" spans="1:6">
+    <row r="392" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
         <v>6</v>
       </c>
@@ -9060,7 +9064,7 @@
         <v>6710</v>
       </c>
     </row>
-    <row r="393" spans="1:6">
+    <row r="393" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
         <v>6</v>
       </c>
@@ -9080,7 +9084,7 @@
         <v>6710</v>
       </c>
     </row>
-    <row r="394" spans="1:6">
+    <row r="394" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
         <v>6</v>
       </c>
@@ -9100,7 +9104,7 @@
         <v>6711</v>
       </c>
     </row>
-    <row r="395" spans="1:6">
+    <row r="395" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
         <v>6</v>
       </c>
@@ -9120,7 +9124,7 @@
         <v>6711</v>
       </c>
     </row>
-    <row r="396" spans="1:6">
+    <row r="396" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
         <v>6</v>
       </c>
@@ -9140,7 +9144,7 @@
         <v>6712</v>
       </c>
     </row>
-    <row r="397" spans="1:6">
+    <row r="397" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
         <v>6</v>
       </c>
@@ -9160,7 +9164,7 @@
         <v>6712</v>
       </c>
     </row>
-    <row r="398" spans="1:6">
+    <row r="398" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
         <v>6</v>
       </c>
@@ -9180,7 +9184,7 @@
         <v>6713</v>
       </c>
     </row>
-    <row r="399" spans="1:6">
+    <row r="399" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
         <v>6</v>
       </c>
@@ -9200,7 +9204,7 @@
         <v>6713</v>
       </c>
     </row>
-    <row r="400" spans="1:6">
+    <row r="400" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
         <v>6</v>
       </c>
@@ -9220,7 +9224,7 @@
         <v>6714</v>
       </c>
     </row>
-    <row r="401" spans="1:6">
+    <row r="401" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
         <v>6</v>
       </c>
@@ -9240,7 +9244,7 @@
         <v>6714</v>
       </c>
     </row>
-    <row r="402" spans="1:6">
+    <row r="402" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
         <v>6</v>
       </c>
@@ -9260,7 +9264,7 @@
         <v>6715</v>
       </c>
     </row>
-    <row r="403" spans="1:6">
+    <row r="403" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
         <v>6</v>
       </c>
@@ -9280,7 +9284,7 @@
         <v>6715</v>
       </c>
     </row>
-    <row r="404" spans="1:6">
+    <row r="404" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
         <v>6</v>
       </c>
@@ -9300,7 +9304,7 @@
         <v>6716</v>
       </c>
     </row>
-    <row r="405" spans="1:6">
+    <row r="405" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
         <v>6</v>
       </c>
@@ -9320,7 +9324,7 @@
         <v>6716</v>
       </c>
     </row>
-    <row r="406" spans="1:6">
+    <row r="406" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
         <v>6</v>
       </c>
@@ -9340,7 +9344,7 @@
         <v>6717</v>
       </c>
     </row>
-    <row r="407" spans="1:6">
+    <row r="407" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
         <v>6</v>
       </c>
@@ -9360,7 +9364,7 @@
         <v>6717</v>
       </c>
     </row>
-    <row r="408" spans="1:6">
+    <row r="408" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
         <v>6</v>
       </c>
@@ -9380,7 +9384,7 @@
         <v>6718</v>
       </c>
     </row>
-    <row r="409" spans="1:6">
+    <row r="409" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
         <v>6</v>
       </c>
@@ -9400,7 +9404,7 @@
         <v>6718</v>
       </c>
     </row>
-    <row r="410" spans="1:6">
+    <row r="410" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
         <v>6</v>
       </c>
@@ -9420,7 +9424,7 @@
         <v>6719</v>
       </c>
     </row>
-    <row r="411" spans="1:6">
+    <row r="411" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
         <v>6</v>
       </c>
@@ -9440,7 +9444,7 @@
         <v>6719</v>
       </c>
     </row>
-    <row r="412" spans="1:6">
+    <row r="412" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
         <v>6</v>
       </c>
@@ -9460,7 +9464,7 @@
         <v>6720</v>
       </c>
     </row>
-    <row r="413" spans="1:6">
+    <row r="413" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
         <v>6</v>
       </c>
@@ -9480,7 +9484,7 @@
         <v>6720</v>
       </c>
     </row>
-    <row r="414" spans="1:6">
+    <row r="414" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
         <v>6</v>
       </c>
@@ -9500,7 +9504,7 @@
         <v>6721</v>
       </c>
     </row>
-    <row r="415" spans="1:6">
+    <row r="415" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
         <v>6</v>
       </c>
@@ -9520,7 +9524,7 @@
         <v>6721</v>
       </c>
     </row>
-    <row r="416" spans="1:6">
+    <row r="416" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
         <v>6</v>
       </c>
@@ -9540,7 +9544,7 @@
         <v>6722</v>
       </c>
     </row>
-    <row r="417" spans="1:6">
+    <row r="417" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
         <v>6</v>
       </c>
@@ -9560,7 +9564,7 @@
         <v>6722</v>
       </c>
     </row>
-    <row r="418" spans="1:6">
+    <row r="418" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
         <v>6</v>
       </c>
@@ -9580,7 +9584,7 @@
         <v>6723</v>
       </c>
     </row>
-    <row r="419" spans="1:6">
+    <row r="419" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
         <v>6</v>
       </c>
@@ -9600,7 +9604,7 @@
         <v>6723</v>
       </c>
     </row>
-    <row r="420" spans="1:6">
+    <row r="420" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
         <v>6</v>
       </c>
@@ -9620,7 +9624,7 @@
         <v>6724</v>
       </c>
     </row>
-    <row r="421" spans="1:6">
+    <row r="421" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
         <v>6</v>
       </c>
@@ -9640,7 +9644,7 @@
         <v>6724</v>
       </c>
     </row>
-    <row r="422" spans="1:6">
+    <row r="422" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
         <v>6</v>
       </c>
@@ -9660,7 +9664,7 @@
         <v>6725</v>
       </c>
     </row>
-    <row r="423" spans="1:6">
+    <row r="423" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
         <v>6</v>
       </c>
@@ -9680,7 +9684,7 @@
         <v>6725</v>
       </c>
     </row>
-    <row r="424" spans="1:6">
+    <row r="424" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
         <v>6</v>
       </c>
@@ -9700,7 +9704,7 @@
         <v>6726</v>
       </c>
     </row>
-    <row r="425" spans="1:6">
+    <row r="425" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
         <v>6</v>
       </c>
@@ -9720,7 +9724,7 @@
         <v>6726</v>
       </c>
     </row>
-    <row r="426" spans="1:6">
+    <row r="426" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
         <v>6</v>
       </c>
@@ -9740,7 +9744,7 @@
         <v>6727</v>
       </c>
     </row>
-    <row r="427" spans="1:6">
+    <row r="427" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
         <v>6</v>
       </c>
@@ -9760,7 +9764,7 @@
         <v>6727</v>
       </c>
     </row>
-    <row r="428" spans="1:6">
+    <row r="428" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
         <v>6</v>
       </c>
@@ -9780,7 +9784,7 @@
         <v>6728</v>
       </c>
     </row>
-    <row r="429" spans="1:6">
+    <row r="429" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
         <v>6</v>
       </c>
@@ -9800,7 +9804,7 @@
         <v>6728</v>
       </c>
     </row>
-    <row r="430" spans="1:6">
+    <row r="430" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
         <v>6</v>
       </c>
@@ -9820,7 +9824,7 @@
         <v>6729</v>
       </c>
     </row>
-    <row r="431" spans="1:6">
+    <row r="431" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
         <v>6</v>
       </c>
@@ -9840,7 +9844,7 @@
         <v>6729</v>
       </c>
     </row>
-    <row r="432" spans="1:6">
+    <row r="432" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
         <v>6</v>
       </c>
@@ -9860,7 +9864,7 @@
         <v>6730</v>
       </c>
     </row>
-    <row r="433" spans="1:6">
+    <row r="433" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
         <v>6</v>
       </c>
@@ -9880,7 +9884,7 @@
         <v>6730</v>
       </c>
     </row>
-    <row r="434" spans="1:6">
+    <row r="434" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
         <v>6</v>
       </c>
@@ -9900,7 +9904,7 @@
         <v>6731</v>
       </c>
     </row>
-    <row r="435" spans="1:6">
+    <row r="435" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
         <v>6</v>
       </c>
@@ -9920,7 +9924,7 @@
         <v>6731</v>
       </c>
     </row>
-    <row r="436" spans="1:6">
+    <row r="436" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
         <v>6</v>
       </c>
@@ -9940,7 +9944,7 @@
         <v>6732</v>
       </c>
     </row>
-    <row r="437" spans="1:6">
+    <row r="437" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
         <v>6</v>
       </c>
@@ -9960,7 +9964,7 @@
         <v>6732</v>
       </c>
     </row>
-    <row r="438" spans="1:6">
+    <row r="438" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
         <v>6</v>
       </c>
@@ -9980,7 +9984,7 @@
         <v>6733</v>
       </c>
     </row>
-    <row r="439" spans="1:6">
+    <row r="439" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
         <v>6</v>
       </c>
@@ -10000,7 +10004,7 @@
         <v>6733</v>
       </c>
     </row>
-    <row r="440" spans="1:6">
+    <row r="440" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
         <v>6</v>
       </c>
@@ -10020,7 +10024,7 @@
         <v>6734</v>
       </c>
     </row>
-    <row r="441" spans="1:6">
+    <row r="441" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
         <v>6</v>
       </c>
@@ -10040,7 +10044,7 @@
         <v>6734</v>
       </c>
     </row>
-    <row r="442" spans="1:6">
+    <row r="442" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
         <v>6</v>
       </c>
@@ -10060,7 +10064,7 @@
         <v>6735</v>
       </c>
     </row>
-    <row r="443" spans="1:6">
+    <row r="443" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
         <v>6</v>
       </c>
@@ -10080,7 +10084,7 @@
         <v>6735</v>
       </c>
     </row>
-    <row r="444" spans="1:6">
+    <row r="444" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
         <v>6</v>
       </c>
@@ -10100,7 +10104,7 @@
         <v>6736</v>
       </c>
     </row>
-    <row r="445" spans="1:6">
+    <row r="445" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
         <v>6</v>
       </c>
@@ -10120,7 +10124,7 @@
         <v>6736</v>
       </c>
     </row>
-    <row r="446" spans="1:6">
+    <row r="446" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
         <v>6</v>
       </c>
@@ -10140,7 +10144,7 @@
         <v>6737</v>
       </c>
     </row>
-    <row r="447" spans="1:6">
+    <row r="447" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
         <v>6</v>
       </c>
@@ -10160,7 +10164,7 @@
         <v>6737</v>
       </c>
     </row>
-    <row r="448" spans="1:6">
+    <row r="448" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
         <v>233</v>
       </c>
@@ -10180,7 +10184,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="449" spans="1:6">
+    <row r="449" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
         <v>233</v>
       </c>
@@ -10200,7 +10204,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="450" spans="1:6">
+    <row r="450" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
         <v>6</v>
       </c>
@@ -10220,7 +10224,7 @@
         <v>6738</v>
       </c>
     </row>
-    <row r="451" spans="1:6">
+    <row r="451" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
         <v>6</v>
       </c>
@@ -10240,7 +10244,7 @@
         <v>6738</v>
       </c>
     </row>
-    <row r="452" spans="1:6">
+    <row r="452" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
         <v>6</v>
       </c>
@@ -10260,7 +10264,7 @@
         <v>6739</v>
       </c>
     </row>
-    <row r="453" spans="1:6">
+    <row r="453" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
         <v>6</v>
       </c>
@@ -10280,7 +10284,7 @@
         <v>6739</v>
       </c>
     </row>
-    <row r="454" spans="1:6">
+    <row r="454" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
         <v>6</v>
       </c>
@@ -10300,7 +10304,7 @@
         <v>6740</v>
       </c>
     </row>
-    <row r="455" spans="1:6">
+    <row r="455" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
         <v>6</v>
       </c>
@@ -10320,7 +10324,7 @@
         <v>6740</v>
       </c>
     </row>
-    <row r="456" spans="1:6">
+    <row r="456" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
         <v>6</v>
       </c>
@@ -10340,7 +10344,7 @@
         <v>6741</v>
       </c>
     </row>
-    <row r="457" spans="1:6">
+    <row r="457" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
         <v>6</v>
       </c>
@@ -10360,7 +10364,7 @@
         <v>6741</v>
       </c>
     </row>
-    <row r="458" spans="1:6">
+    <row r="458" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
         <v>6</v>
       </c>
@@ -10380,7 +10384,7 @@
         <v>6742</v>
       </c>
     </row>
-    <row r="459" spans="1:6">
+    <row r="459" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
         <v>6</v>
       </c>
@@ -10400,7 +10404,7 @@
         <v>6742</v>
       </c>
     </row>
-    <row r="460" spans="1:6">
+    <row r="460" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
         <v>6</v>
       </c>
@@ -10420,7 +10424,7 @@
         <v>6743</v>
       </c>
     </row>
-    <row r="461" spans="1:6">
+    <row r="461" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
         <v>6</v>
       </c>
@@ -10440,7 +10444,7 @@
         <v>6743</v>
       </c>
     </row>
-    <row r="462" spans="1:6">
+    <row r="462" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
         <v>6</v>
       </c>
@@ -10460,7 +10464,7 @@
         <v>6744</v>
       </c>
     </row>
-    <row r="463" spans="1:6">
+    <row r="463" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
         <v>6</v>
       </c>
@@ -10480,7 +10484,7 @@
         <v>6744</v>
       </c>
     </row>
-    <row r="464" spans="1:6">
+    <row r="464" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
         <v>6</v>
       </c>
@@ -10500,7 +10504,7 @@
         <v>6745</v>
       </c>
     </row>
-    <row r="465" spans="1:6">
+    <row r="465" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
         <v>6</v>
       </c>
@@ -10520,7 +10524,7 @@
         <v>6745</v>
       </c>
     </row>
-    <row r="466" spans="1:6">
+    <row r="466" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
         <v>6</v>
       </c>
@@ -10540,7 +10544,7 @@
         <v>6746</v>
       </c>
     </row>
-    <row r="467" spans="1:6">
+    <row r="467" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
         <v>6</v>
       </c>
@@ -10560,7 +10564,7 @@
         <v>6746</v>
       </c>
     </row>
-    <row r="468" spans="1:6">
+    <row r="468" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
         <v>6</v>
       </c>
@@ -10580,7 +10584,7 @@
         <v>6747</v>
       </c>
     </row>
-    <row r="469" spans="1:6">
+    <row r="469" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
         <v>6</v>
       </c>
@@ -10600,7 +10604,7 @@
         <v>6747</v>
       </c>
     </row>
-    <row r="470" spans="1:6">
+    <row r="470" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
         <v>6</v>
       </c>
@@ -10620,7 +10624,7 @@
         <v>6748</v>
       </c>
     </row>
-    <row r="471" spans="1:6">
+    <row r="471" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
         <v>6</v>
       </c>
@@ -10640,7 +10644,7 @@
         <v>6748</v>
       </c>
     </row>
-    <row r="472" spans="1:6">
+    <row r="472" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
         <v>6</v>
       </c>
@@ -10660,7 +10664,7 @@
         <v>6749</v>
       </c>
     </row>
-    <row r="473" spans="1:6">
+    <row r="473" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
         <v>6</v>
       </c>
@@ -10680,7 +10684,7 @@
         <v>6749</v>
       </c>
     </row>
-    <row r="474" spans="1:6">
+    <row r="474" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
         <v>6</v>
       </c>
@@ -10700,7 +10704,7 @@
         <v>6750</v>
       </c>
     </row>
-    <row r="475" spans="1:6">
+    <row r="475" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
         <v>6</v>
       </c>
@@ -10720,7 +10724,7 @@
         <v>6750</v>
       </c>
     </row>
-    <row r="476" spans="1:6">
+    <row r="476" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
         <v>6</v>
       </c>
@@ -10740,7 +10744,7 @@
         <v>6751</v>
       </c>
     </row>
-    <row r="477" spans="1:6">
+    <row r="477" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
         <v>6</v>
       </c>
@@ -10760,7 +10764,7 @@
         <v>6751</v>
       </c>
     </row>
-    <row r="478" spans="1:6">
+    <row r="478" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
         <v>6</v>
       </c>
@@ -10780,7 +10784,7 @@
         <v>6752</v>
       </c>
     </row>
-    <row r="479" spans="1:6">
+    <row r="479" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
         <v>6</v>
       </c>
@@ -10800,7 +10804,7 @@
         <v>6752</v>
       </c>
     </row>
-    <row r="480" spans="1:6">
+    <row r="480" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
         <v>6</v>
       </c>
@@ -10820,7 +10824,7 @@
         <v>6753</v>
       </c>
     </row>
-    <row r="481" spans="1:6">
+    <row r="481" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
         <v>6</v>
       </c>
@@ -10840,7 +10844,7 @@
         <v>6753</v>
       </c>
     </row>
-    <row r="482" spans="1:6">
+    <row r="482" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A482" t="s">
         <v>6</v>
       </c>
@@ -10860,7 +10864,7 @@
         <v>6754</v>
       </c>
     </row>
-    <row r="483" spans="1:6">
+    <row r="483" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A483" t="s">
         <v>6</v>
       </c>
@@ -10880,7 +10884,7 @@
         <v>6754</v>
       </c>
     </row>
-    <row r="484" spans="1:6">
+    <row r="484" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
         <v>6</v>
       </c>
@@ -10900,7 +10904,7 @@
         <v>6755</v>
       </c>
     </row>
-    <row r="485" spans="1:6">
+    <row r="485" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A485" t="s">
         <v>6</v>
       </c>
@@ -10920,7 +10924,7 @@
         <v>6755</v>
       </c>
     </row>
-    <row r="486" spans="1:6">
+    <row r="486" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
         <v>6</v>
       </c>
@@ -10940,7 +10944,7 @@
         <v>6756</v>
       </c>
     </row>
-    <row r="487" spans="1:6">
+    <row r="487" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
         <v>6</v>
       </c>
@@ -10960,7 +10964,7 @@
         <v>6756</v>
       </c>
     </row>
-    <row r="488" spans="1:6">
+    <row r="488" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
         <v>6</v>
       </c>
@@ -10980,7 +10984,7 @@
         <v>6757</v>
       </c>
     </row>
-    <row r="489" spans="1:6">
+    <row r="489" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
         <v>6</v>
       </c>
@@ -11000,7 +11004,7 @@
         <v>6757</v>
       </c>
     </row>
-    <row r="490" spans="1:6">
+    <row r="490" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
         <v>6</v>
       </c>
@@ -11020,7 +11024,7 @@
         <v>6758</v>
       </c>
     </row>
-    <row r="491" spans="1:6">
+    <row r="491" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
         <v>6</v>
       </c>
@@ -11040,7 +11044,7 @@
         <v>6758</v>
       </c>
     </row>
-    <row r="492" spans="1:6">
+    <row r="492" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A492" t="s">
         <v>6</v>
       </c>
@@ -11060,7 +11064,7 @@
         <v>6759</v>
       </c>
     </row>
-    <row r="493" spans="1:6">
+    <row r="493" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A493" t="s">
         <v>6</v>
       </c>
@@ -11080,7 +11084,7 @@
         <v>6759</v>
       </c>
     </row>
-    <row r="494" spans="1:6">
+    <row r="494" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
         <v>6</v>
       </c>
@@ -11100,7 +11104,7 @@
         <v>6760</v>
       </c>
     </row>
-    <row r="495" spans="1:6">
+    <row r="495" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A495" t="s">
         <v>6</v>
       </c>
@@ -11120,7 +11124,7 @@
         <v>6760</v>
       </c>
     </row>
-    <row r="496" spans="1:6">
+    <row r="496" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A496" t="s">
         <v>6</v>
       </c>
@@ -11140,7 +11144,7 @@
         <v>6761</v>
       </c>
     </row>
-    <row r="497" spans="1:6">
+    <row r="497" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A497" t="s">
         <v>6</v>
       </c>
@@ -11160,7 +11164,7 @@
         <v>6761</v>
       </c>
     </row>
-    <row r="498" spans="1:6">
+    <row r="498" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A498" t="s">
         <v>6</v>
       </c>
@@ -11180,7 +11184,7 @@
         <v>6762</v>
       </c>
     </row>
-    <row r="499" spans="1:6">
+    <row r="499" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A499" t="s">
         <v>6</v>
       </c>
@@ -11200,7 +11204,7 @@
         <v>6762</v>
       </c>
     </row>
-    <row r="500" spans="1:6">
+    <row r="500" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A500" t="s">
         <v>6</v>
       </c>
@@ -11220,7 +11224,7 @@
         <v>6763</v>
       </c>
     </row>
-    <row r="501" spans="1:6">
+    <row r="501" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A501" t="s">
         <v>6</v>
       </c>
@@ -11240,7 +11244,7 @@
         <v>6763</v>
       </c>
     </row>
-    <row r="502" spans="1:6">
+    <row r="502" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A502" t="s">
         <v>6</v>
       </c>
@@ -11260,7 +11264,7 @@
         <v>6764</v>
       </c>
     </row>
-    <row r="503" spans="1:6">
+    <row r="503" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A503" t="s">
         <v>6</v>
       </c>
@@ -11280,7 +11284,7 @@
         <v>6764</v>
       </c>
     </row>
-    <row r="504" spans="1:6">
+    <row r="504" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A504" t="s">
         <v>6</v>
       </c>
@@ -11300,7 +11304,7 @@
         <v>6765</v>
       </c>
     </row>
-    <row r="505" spans="1:6">
+    <row r="505" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A505" t="s">
         <v>6</v>
       </c>
@@ -11320,7 +11324,7 @@
         <v>6765</v>
       </c>
     </row>
-    <row r="506" spans="1:6">
+    <row r="506" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A506" t="s">
         <v>6</v>
       </c>
@@ -11340,7 +11344,7 @@
         <v>6766</v>
       </c>
     </row>
-    <row r="507" spans="1:6">
+    <row r="507" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A507" t="s">
         <v>6</v>
       </c>
@@ -11360,7 +11364,7 @@
         <v>6766</v>
       </c>
     </row>
-    <row r="508" spans="1:6">
+    <row r="508" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A508" t="s">
         <v>6</v>
       </c>
@@ -11380,7 +11384,7 @@
         <v>6767</v>
       </c>
     </row>
-    <row r="509" spans="1:6">
+    <row r="509" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A509" t="s">
         <v>6</v>
       </c>
@@ -11400,7 +11404,7 @@
         <v>6767</v>
       </c>
     </row>
-    <row r="510" spans="1:6">
+    <row r="510" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A510" t="s">
         <v>6</v>
       </c>
@@ -11420,7 +11424,7 @@
         <v>6768</v>
       </c>
     </row>
-    <row r="511" spans="1:6">
+    <row r="511" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A511" t="s">
         <v>6</v>
       </c>
@@ -11446,26 +11450,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="2b8f46f0-82da-4ef7-969d-ac4cdf93ac59" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="06af1c99-a7ef-4c15-a896-fa313c6850d6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008726E51B410DEB45AC78922F1F642D3F" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d816f4804f51798b5fbcf5439326a0dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="06af1c99-a7ef-4c15-a896-fa313c6850d6" xmlns:ns3="2b8f46f0-82da-4ef7-969d-ac4cdf93ac59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7ca303054d7b5d5b0935165f9e4aa098" ns2:_="" ns3:_="">
     <xsd:import namespace="06af1c99-a7ef-4c15-a896-fa313c6850d6"/>
@@ -11660,14 +11644,60 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="2b8f46f0-82da-4ef7-969d-ac4cdf93ac59" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="06af1c99-a7ef-4c15-a896-fa313c6850d6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A9C502-E846-4EDC-A62B-44810CD5FF45}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A740393-D650-4713-848F-8569228BC5AA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="06af1c99-a7ef-4c15-a896-fa313c6850d6"/>
+    <ds:schemaRef ds:uri="2b8f46f0-82da-4ef7-969d-ac4cdf93ac59"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9CFA68FA-10C2-4395-92C8-EF3A7DE884B4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A9C502-E846-4EDC-A62B-44810CD5FF45}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2b8f46f0-82da-4ef7-969d-ac4cdf93ac59"/>
+    <ds:schemaRef ds:uri="06af1c99-a7ef-4c15-a896-fa313c6850d6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A740393-D650-4713-848F-8569228BC5AA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9CFA68FA-10C2-4395-92C8-EF3A7DE884B4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>